<commit_message>
New screenshots and Store images; record the 0.5.0 release
Wider windows so the toolbar is not crowded, sample files that read like real documents (a newsletter in Segoe UI with real tables, a budget with charts, a presentation, trip notes in the dark theme), captured only after each file has opened. The Store logo (300 x 300) and four Store screenshots are in docs/images/store; the README shows the four screenshots.
</commit_message>
<xml_diff>
--- a/docs/images/showcase/Household budget.xlsx
+++ b/docs/images/showcase/Household budget.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>Household budget 2026</t>
   </si>
@@ -54,9 +54,6 @@
   </si>
   <si>
     <t>Other</t>
-  </si>
-  <si>
-    <t>Values are the saved results: Plain Viewer never recalculates formulas.</t>
   </si>
   <si>
     <t>Budget notes</t>
@@ -72,7 +69,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -91,10 +88,6 @@
     </font>
     <font>
       <b/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF6B7280"/>
     </font>
   </fonts>
   <fills count="4">
@@ -134,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -150,7 +143,6 @@
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -167,6 +159,479 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:r>
+              <a:t>Monthly spending that changes</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Budget 2026'!$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Groceries</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2563EB"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Budget 2026'!$B$3:$E$3</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>January</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>February</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>March</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>April</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Budget 2026'!$B$5:$E$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>412.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>389.2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>430.75</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>405.1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Budget 2026'!$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Electricity and gas</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="F59E0B"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Budget 2026'!$B$3:$E$3</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>January</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>February</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>March</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>April</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Budget 2026'!$B$6:$E$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>138.4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>126.9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>101.3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>84.6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Budget 2026'!$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Transport</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="10B981"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Budget 2026'!$B$3:$E$3</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>January</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>February</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>March</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>April</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Budget 2026'!$B$8:$E$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>96</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>88.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>102</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>94.25</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Budget 2026'!$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Other</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="8B5CF6"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Budget 2026'!$B$3:$E$3</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>January</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>February</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>March</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>April</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Budget 2026'!$B$10:$E$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>64.9</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>88</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:overlap val="100"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:crossAx val="2"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:crossAx val="1"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:r>
+              <a:t>Where the money went</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Budget 2026'!$F$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Budget 2026'!$A$4:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>Rent</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Groceries</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Electricity and gas</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Internet and phone</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Transport</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Savings</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Other</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Budget 2026'!$F$4:$F$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>3800</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1637.55</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>451.2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>380.75</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1300</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>318.4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="50"/>
+      </c:doughnutChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Monthly spending"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Where the money went"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -491,7 +956,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -701,17 +1166,13 @@
         <v>8107.9</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
-        <v>14</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rIdShowcaseDrawing"/>
 </worksheet>
 </file>
 
@@ -721,13 +1182,13 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
-        <v>15</v>
+      <c r="A1" s="11" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>